<commit_message>
docs(kiểm-toán): Chuẩn hóa số liệu độ phủ, cập nhật hash bằng chứng và hoàn thiện báo cáo độc lập cuối cùng
- Hoàn thành rà soát độc lập cuối cùng 10 công đoạn theo yêu cầu nghiệm thu.
- Xác nhận bản vá v1 áp dụng chính xác và độc lập lên baseline 44202070c68002d9af068374478cdc83098dd4d8, 17/17 smoke tests PASS.
- Chuẩn hóa tỷ lệ độ phủ dòng lệnh chính xác từ gcovr: 45.84% (353/770 lines), nhánh 36.02% trên source/src/.
- Đồng bộ hóa 100% mã băm SHA256 thật từ 28 tập tin log vào evidence_manifest.csv và các workbook.
- Xuất bản tài liệu kiểm toán độc lập chi tiết: docs/09_Final_Report/FINAL_INDEPENDENT_AUDIT.md.
</commit_message>
<xml_diff>
--- a/docs/07_CWE_Coverage/coverage_report.xlsx
+++ b/docs/07_CWE_Coverage/coverage_report.xlsx
@@ -509,16 +509,16 @@
         <v>100</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>87.0%</t>
+          <t>81.0%</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>78.5%</t>
+          <t>56.5% (52/92)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -528,7 +528,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Các nhánh I/O lỗi phần cứng hiếm gặp (fputs fail)</t>
+          <t>Các nhánh I/O lỗi phần cứng (fputs fail)</t>
         </is>
       </c>
     </row>
@@ -542,21 +542,21 @@
         <v>43</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>88.4%</t>
+          <t>67.4%</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>82.1%</t>
+          <t>41.7% (10/24)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Phủ toàn bộ import_stock, export_stock, find_product, inventory_free</t>
+          <t>Phủ import_stock, export_stock, find_product, inventory_free</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -575,26 +575,26 @@
         <v>135</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>60.7%</t>
+          <t>76.3%</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>55.0%</t>
+          <t>55.3% (63/114)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Phủ init, add_product, realloc growth, delete_product, find_product_by_id</t>
+          <t>Phủ product_list_init, add_product, realloc growth, delete_product, find_product_by_id</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Nhánh so sánh chuỗi không phân biệt hoa thường trong search_name</t>
+          <t>Nhánh so sánh chuỗi trong search_name</t>
         </is>
       </c>
     </row>
@@ -608,26 +608,26 @@
         <v>204</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>34.3%</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>29.5% (33/112)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Phủ tính toán tóm tắt nhóm hàng cơ bản trong smoke test</t>
+          <t>Phủ tóm tắt nhóm hàng cơ bản trong smoke test</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Giao diện in ấn báo cáo bảng CLI rộng (không thuộc luồng kiểm toán cốt lõi)</t>
+          <t>Giao diện in báo cáo bảng CLI rộng</t>
         </is>
       </c>
     </row>
@@ -641,26 +641,26 @@
         <v>123</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>28.5%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>9.1% (10/110)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Phủ safe_string_copy, trim_whitespace, parse helpers</t>
+          <t>Phủ safe_string_copy, trim_whitespace</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Các hàm tiện ích phụ trợ chuyển đổi chuỗi chưa gọi trong luồng nhập kho</t>
+          <t>Các tiện ích phụ trợ chuyển đổi chuỗi chưa gọi trong luồng nhập kho</t>
         </is>
       </c>
     </row>
@@ -674,16 +674,16 @@
         <v>165</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>51.5%</t>
+          <t>33.3%</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>46.0%</t>
+          <t>32.7% (51/156)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -700,33 +700,33 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TỔNG CỘNG HỆ THỐNG</t>
+          <t>TỔNG CỘNG MÃ NGUỒN C (source/src/)</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
         <v>770</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>46.1%</t>
+          <t>45.84%</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>41.5%</t>
+          <t>36.02% (219/608)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Tăng từ 36.4% lên 46.1% nhờ bổ sung 6 bộ test driver mô phỏng C</t>
+          <t>Tăng từ 36.4% ở Bước 3 lên 45.84% dòng và 36.02% nhánh nhờ 6 bộ C Simulator</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Các module report và menu CLI không bắt buộc phải phủ 100%</t>
+          <t>Module report và CLI không bắt buộc phủ 100% trong luồng kiểm toán</t>
         </is>
       </c>
     </row>

</xml_diff>